<commit_message>
daily auto-refresh 2026-10-05 13:00
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,427 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:G17"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>438</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>60</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>85.7</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17013</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>256</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18189</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>441</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>432</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2671</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>294</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.09999999999999</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>211705</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>581</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>568</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3505</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>347</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>61.1</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>40966</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>640</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>629</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>3862</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>344</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>54.7</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>83257</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>436</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>431</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>2638</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>258</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>59.9</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>23298</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>838</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>811</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>5545</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>450</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>55.5</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>46341</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>883</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>821</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>6624</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>633</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>77.09999999999999</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>62836</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1545</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1486</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>10168</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1241</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>83.5</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>211790</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>993</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>877</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>6031</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>762</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>86.90000000000001</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>140500</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1139</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>587</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6945</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>511</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>87.09999999999999</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>72216</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3814</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>3026</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>23425</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2091</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>69.09999999999999</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>48803</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>3030</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>2368</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>17922</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1007</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>42.5</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>41153</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2415</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>847</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>13017</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>429</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>50.6</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>19251</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1238</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>508</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>7483</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>171</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>33.7</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>7447</v>
       </c>
     </row>
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>154</v>
+      </c>
+      <c r="C17">
+        <v>70</v>
+      </c>
+      <c r="D17">
+        <v>801</v>
+      </c>
+      <c r="E17">
+        <v>0</v>
+      </c>
+      <c r="F17">
+        <v>0</v>
+      </c>
+      <c r="G17">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-09 15:06
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -475,7 +475,7 @@
         <v>85.7</v>
       </c>
       <c r="G2" t="n">
-        <v>17018</v>
+        <v>17004</v>
       </c>
     </row>
     <row r="3">
@@ -525,7 +525,7 @@
         <v>68.09999999999999</v>
       </c>
       <c r="G4" t="n">
-        <v>213208</v>
+        <v>213297</v>
       </c>
     </row>
     <row r="5">
@@ -550,7 +550,7 @@
         <v>61.1</v>
       </c>
       <c r="G5" t="n">
-        <v>41510</v>
+        <v>41509</v>
       </c>
     </row>
     <row r="6">
@@ -575,7 +575,7 @@
         <v>54.7</v>
       </c>
       <c r="G6" t="n">
-        <v>83325</v>
+        <v>83335</v>
       </c>
     </row>
     <row r="7">
@@ -650,7 +650,7 @@
         <v>77.09999999999999</v>
       </c>
       <c r="G9" t="n">
-        <v>64139</v>
+        <v>64077</v>
       </c>
     </row>
     <row r="10">
@@ -675,7 +675,7 @@
         <v>83.59999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>216640</v>
+        <v>216446</v>
       </c>
     </row>
     <row r="11">
@@ -700,7 +700,7 @@
         <v>86.90000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>142859</v>
+        <v>142813</v>
       </c>
     </row>
     <row r="12">
@@ -725,7 +725,7 @@
         <v>87.09999999999999</v>
       </c>
       <c r="G12" t="n">
-        <v>72534</v>
+        <v>72160</v>
       </c>
     </row>
     <row r="13">
@@ -750,7 +750,7 @@
         <v>68.8</v>
       </c>
       <c r="G13" t="n">
-        <v>51994</v>
+        <v>52159</v>
       </c>
     </row>
     <row r="14">
@@ -769,13 +769,13 @@
         <v>17922</v>
       </c>
       <c r="E14" t="n">
-        <v>881</v>
+        <v>862</v>
       </c>
       <c r="F14" t="n">
-        <v>37.2</v>
+        <v>36.4</v>
       </c>
       <c r="G14" t="n">
-        <v>38618</v>
+        <v>37607</v>
       </c>
     </row>
     <row r="15">
@@ -794,13 +794,13 @@
         <v>13012</v>
       </c>
       <c r="E15" t="n">
-        <v>429</v>
+        <v>428</v>
       </c>
       <c r="F15" t="n">
-        <v>50.6</v>
+        <v>50.5</v>
       </c>
       <c r="G15" t="n">
-        <v>21987</v>
+        <v>22068</v>
       </c>
     </row>
     <row r="16">
@@ -819,13 +819,13 @@
         <v>7477</v>
       </c>
       <c r="E16" t="n">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F16" t="n">
-        <v>44.8</v>
+        <v>45.4</v>
       </c>
       <c r="G16" t="n">
-        <v>11121</v>
+        <v>11312</v>
       </c>
     </row>
     <row r="17">
@@ -844,10 +844,10 @@
         <v>2526</v>
       </c>
       <c r="E17" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F17" t="n">
-        <v>7.4</v>
+        <v>10.1</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 09:30
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,452 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>415</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>60</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>85.7</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17509</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>243</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18234</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>441</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>432</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2533</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>297</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>214487</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>581</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>568</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3324</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>354</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>62.3</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>42818</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>640</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>629</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>3663</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>348</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>55.3</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>84416</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>436</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>431</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>2502</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>259</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>60.1</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>23749</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>838</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>812</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>5286</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>458</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>56.4</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>47229</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>883</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>821</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>6405</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>646</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>78.7</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>64063</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1545</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1486</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>9711</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1272</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>85.59999999999999</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>216996</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>993</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>877</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>5726</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>777</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>88.59999999999999</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>140785</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1139</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>587</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6529</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>517</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>88.09999999999999</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>71064</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3814</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>3026</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>22166</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2154</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>71.2</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>51541</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>3030</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>2368</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>17252</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1251</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>52.8</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>39103</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2415</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>847</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>19275</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>460</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>54.3</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>23873</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1237</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>511</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>7451</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>294</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>57.5</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>13174</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
         <v>2715</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>1012</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17">
         <v>19158</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>204</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17">
         <v>20.2</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17">
         <v>614</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 09:32
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,120 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>sample_orders</t>
-  </si>
-  <si>
-    <t>new_creators</t>
-  </si>
-  <si>
-    <t>cogs</t>
-  </si>
-  <si>
-    <t>posted</t>
-  </si>
-  <si>
-    <t>post_rate</t>
-  </si>
-  <si>
-    <t>video_gmv</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
-  </si>
-  <si>
-    <t>2026-01</t>
-  </si>
-  <si>
-    <t>2026-02</t>
-  </si>
-  <si>
-    <t>2026-03</t>
-  </si>
-  <si>
-    <t>2026-04</t>
-  </si>
-  <si>
-    <t>2026-05</t>
-  </si>
-  <si>
-    <t>2026-06</t>
-  </si>
-  <si>
-    <t>2026-07</t>
-  </si>
-  <si>
-    <t>2026-08</t>
-  </si>
-  <si>
-    <t>2026-09</t>
-  </si>
-  <si>
-    <t>2026-10</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -122,36 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -439,402 +408,452 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sample_orders</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>new_creators</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cogs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>posted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>post_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>video_gmv</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>73</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>70</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>415</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>60</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>85.7</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>17509</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>42</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>41</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>243</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>33</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>80.5</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>18234</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>441</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>432</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>2533</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>297</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>68.8</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>214487</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>581</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>568</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>3324</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>354</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>62.3</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>42818</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>640</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>629</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>3663</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>348</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>55.3</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>84416</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>436</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>431</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>2502</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>259</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>60.1</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>23749</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>838</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>812</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>5286</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>458</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>56.4</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>47229</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>883</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>821</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>6405</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>646</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>78.7</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>64063</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>1545</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>1486</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>9711</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>1272</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>85.59999999999999</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>216996</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>993</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>877</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>5726</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>777</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>88.59999999999999</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>140785</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1139</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="n">
         <v>587</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>6529</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>517</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>88.09999999999999</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="n">
         <v>71064</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>3814</v>
       </c>
-      <c r="C13">
+      <c r="C13" t="n">
         <v>3026</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>22166</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>2154</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>71.2</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>51541</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>3030</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="n">
         <v>2368</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>17252</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>1251</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>52.8</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>39103</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>2415</v>
       </c>
-      <c r="C15">
+      <c r="C15" t="n">
         <v>847</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>19275</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>460</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>54.3</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>23873</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>1237</v>
       </c>
-      <c r="C16">
+      <c r="C16" t="n">
         <v>511</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>7451</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>294</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="n">
         <v>57.5</v>
       </c>
-      <c r="G16">
+      <c r="G16" t="n">
         <v>13174</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>2715</v>
       </c>
-      <c r="C17">
+      <c r="C17" t="n">
         <v>1012</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="n">
         <v>19158</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="n">
         <v>204</v>
       </c>
-      <c r="F17">
+      <c r="F17" t="n">
         <v>20.2</v>
       </c>
-      <c r="G17">
+      <c r="G17" t="n">
         <v>614</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 11:19
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,452 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>415</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>60</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>85.7</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17509</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>243</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18234</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>441</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>432</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2533</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>297</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>214487</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>581</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>568</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3324</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>354</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>62.3</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>42818</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>640</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>629</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>3663</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>348</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>55.3</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>84416</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>436</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>431</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>2502</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>259</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>60.1</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>23749</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>838</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>812</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>5286</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>458</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>56.4</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>47229</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>883</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>821</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>6405</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>646</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>78.7</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>64063</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1545</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1486</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>9711</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1272</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>85.59999999999999</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>216996</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>993</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>877</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>5726</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>777</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>88.59999999999999</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>140785</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1139</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>587</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6529</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>517</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>88.09999999999999</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>71064</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3814</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>3026</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>22166</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2154</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>71.2</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>51541</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>3030</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>2368</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>17252</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1251</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>52.8</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>39103</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2415</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>847</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>19275</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>460</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>54.3</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>23873</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1237</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>511</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>7451</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>294</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>57.5</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>13174</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
         <v>2715</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>1012</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17">
         <v>19158</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>204</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17">
         <v>20.2</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17">
         <v>614</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 14:40
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -480,13 +480,13 @@
         <v>415</v>
       </c>
       <c r="E2">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F2">
-        <v>85.7</v>
+        <v>84.3</v>
       </c>
       <c r="G2">
-        <v>17509</v>
+        <v>17413</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -532,7 +532,7 @@
         <v>68.8</v>
       </c>
       <c r="G4">
-        <v>214487</v>
+        <v>214540</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -555,7 +555,7 @@
         <v>62.3</v>
       </c>
       <c r="G5">
-        <v>42818</v>
+        <v>42817</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -578,7 +578,7 @@
         <v>55.3</v>
       </c>
       <c r="G6">
-        <v>84416</v>
+        <v>84414</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -586,22 +586,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="C7">
-        <v>431</v>
+        <v>429</v>
       </c>
       <c r="D7">
-        <v>2502</v>
+        <v>2490</v>
       </c>
       <c r="E7">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="F7">
         <v>60.1</v>
       </c>
       <c r="G7">
-        <v>23749</v>
+        <v>23796</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -624,7 +624,7 @@
         <v>56.4</v>
       </c>
       <c r="G8">
-        <v>47229</v>
+        <v>47228</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -647,7 +647,7 @@
         <v>78.7</v>
       </c>
       <c r="G9">
-        <v>64063</v>
+        <v>64128</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -655,13 +655,13 @@
         <v>15</v>
       </c>
       <c r="B10">
-        <v>1545</v>
+        <v>1543</v>
       </c>
       <c r="C10">
         <v>1486</v>
       </c>
       <c r="D10">
-        <v>9711</v>
+        <v>9700</v>
       </c>
       <c r="E10">
         <v>1272</v>
@@ -670,7 +670,7 @@
         <v>85.59999999999999</v>
       </c>
       <c r="G10">
-        <v>216996</v>
+        <v>217154</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -678,22 +678,22 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>993</v>
+        <v>991</v>
       </c>
       <c r="C11">
-        <v>877</v>
+        <v>876</v>
       </c>
       <c r="D11">
-        <v>5726</v>
+        <v>5715</v>
       </c>
       <c r="E11">
         <v>777</v>
       </c>
       <c r="F11">
-        <v>88.59999999999999</v>
+        <v>88.7</v>
       </c>
       <c r="G11">
-        <v>140785</v>
+        <v>138961</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -701,22 +701,22 @@
         <v>17</v>
       </c>
       <c r="B12">
-        <v>1139</v>
+        <v>1122</v>
       </c>
       <c r="C12">
-        <v>587</v>
+        <v>571</v>
       </c>
       <c r="D12">
-        <v>6529</v>
+        <v>6524</v>
       </c>
       <c r="E12">
         <v>517</v>
       </c>
       <c r="F12">
-        <v>88.09999999999999</v>
+        <v>90.5</v>
       </c>
       <c r="G12">
-        <v>71064</v>
+        <v>71156</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -724,22 +724,22 @@
         <v>18</v>
       </c>
       <c r="B13">
-        <v>3814</v>
+        <v>3753</v>
       </c>
       <c r="C13">
-        <v>3026</v>
+        <v>2975</v>
       </c>
       <c r="D13">
-        <v>22166</v>
+        <v>21939</v>
       </c>
       <c r="E13">
-        <v>2154</v>
+        <v>2149</v>
       </c>
       <c r="F13">
-        <v>71.2</v>
+        <v>72.2</v>
       </c>
       <c r="G13">
-        <v>51541</v>
+        <v>51505</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -747,22 +747,22 @@
         <v>19</v>
       </c>
       <c r="B14">
-        <v>3030</v>
+        <v>2402</v>
       </c>
       <c r="C14">
-        <v>2368</v>
+        <v>1760</v>
       </c>
       <c r="D14">
-        <v>17252</v>
+        <v>14293</v>
       </c>
       <c r="E14">
-        <v>1251</v>
+        <v>1235</v>
       </c>
       <c r="F14">
-        <v>52.8</v>
+        <v>70.2</v>
       </c>
       <c r="G14">
-        <v>39103</v>
+        <v>37088</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -770,22 +770,22 @@
         <v>20</v>
       </c>
       <c r="B15">
-        <v>2415</v>
+        <v>2077</v>
       </c>
       <c r="C15">
-        <v>847</v>
+        <v>519</v>
       </c>
       <c r="D15">
-        <v>19275</v>
+        <v>17453</v>
       </c>
       <c r="E15">
-        <v>460</v>
+        <v>447</v>
       </c>
       <c r="F15">
-        <v>54.3</v>
+        <v>86.09999999999999</v>
       </c>
       <c r="G15">
-        <v>23873</v>
+        <v>23899</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -793,22 +793,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>1237</v>
+        <v>1039</v>
       </c>
       <c r="C16">
-        <v>511</v>
+        <v>331</v>
       </c>
       <c r="D16">
-        <v>7451</v>
+        <v>6274</v>
       </c>
       <c r="E16">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="F16">
-        <v>57.5</v>
+        <v>87.3</v>
       </c>
       <c r="G16">
-        <v>13174</v>
+        <v>13188</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -816,22 +816,22 @@
         <v>22</v>
       </c>
       <c r="B17">
-        <v>2715</v>
+        <v>2549</v>
       </c>
       <c r="C17">
-        <v>1012</v>
+        <v>871</v>
       </c>
       <c r="D17">
-        <v>19158</v>
+        <v>18216</v>
       </c>
       <c r="E17">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="F17">
-        <v>20.2</v>
+        <v>23.3</v>
       </c>
       <c r="G17">
-        <v>614</v>
+        <v>639</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 20:14
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -693,7 +693,7 @@
         <v>88.7</v>
       </c>
       <c r="G11">
-        <v>138961</v>
+        <v>138970</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -716,7 +716,7 @@
         <v>90.5</v>
       </c>
       <c r="G12">
-        <v>71156</v>
+        <v>71155</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -762,7 +762,7 @@
         <v>70.2</v>
       </c>
       <c r="G14">
-        <v>37088</v>
+        <v>37127</v>
       </c>
     </row>
     <row r="15" spans="1:7">

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-22 20:25
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -517,22 +517,22 @@
         <v>9</v>
       </c>
       <c r="B4">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="C4">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="D4">
-        <v>2533</v>
+        <v>2539</v>
       </c>
       <c r="E4">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F4">
         <v>68.8</v>
       </c>
       <c r="G4">
-        <v>214540</v>
+        <v>214753</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -540,22 +540,22 @@
         <v>10</v>
       </c>
       <c r="B5">
-        <v>581</v>
+        <v>662</v>
       </c>
       <c r="C5">
-        <v>568</v>
+        <v>605</v>
       </c>
       <c r="D5">
-        <v>3324</v>
+        <v>3865</v>
       </c>
       <c r="E5">
-        <v>354</v>
+        <v>386</v>
       </c>
       <c r="F5">
-        <v>62.3</v>
+        <v>63.8</v>
       </c>
       <c r="G5">
-        <v>42817</v>
+        <v>46738</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -563,22 +563,22 @@
         <v>11</v>
       </c>
       <c r="B6">
-        <v>640</v>
+        <v>765</v>
       </c>
       <c r="C6">
-        <v>629</v>
+        <v>715</v>
       </c>
       <c r="D6">
-        <v>3663</v>
+        <v>4498</v>
       </c>
       <c r="E6">
-        <v>348</v>
+        <v>421</v>
       </c>
       <c r="F6">
-        <v>55.3</v>
+        <v>58.9</v>
       </c>
       <c r="G6">
-        <v>84414</v>
+        <v>85640</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -586,22 +586,22 @@
         <v>12</v>
       </c>
       <c r="B7">
-        <v>434</v>
+        <v>531</v>
       </c>
       <c r="C7">
-        <v>429</v>
+        <v>491</v>
       </c>
       <c r="D7">
-        <v>2490</v>
+        <v>3138</v>
       </c>
       <c r="E7">
-        <v>258</v>
+        <v>313</v>
       </c>
       <c r="F7">
-        <v>60.1</v>
+        <v>63.7</v>
       </c>
       <c r="G7">
-        <v>23796</v>
+        <v>27811</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -609,22 +609,22 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>838</v>
+        <v>979</v>
       </c>
       <c r="C8">
-        <v>812</v>
+        <v>924</v>
       </c>
       <c r="D8">
-        <v>5286</v>
+        <v>6589</v>
       </c>
       <c r="E8">
-        <v>458</v>
+        <v>546</v>
       </c>
       <c r="F8">
-        <v>56.4</v>
+        <v>59.1</v>
       </c>
       <c r="G8">
-        <v>47228</v>
+        <v>62714</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -632,22 +632,22 @@
         <v>14</v>
       </c>
       <c r="B9">
-        <v>883</v>
+        <v>1113</v>
       </c>
       <c r="C9">
-        <v>821</v>
+        <v>997</v>
       </c>
       <c r="D9">
-        <v>6405</v>
+        <v>9651</v>
       </c>
       <c r="E9">
-        <v>646</v>
+        <v>788</v>
       </c>
       <c r="F9">
-        <v>78.7</v>
+        <v>79</v>
       </c>
       <c r="G9">
-        <v>64128</v>
+        <v>67642</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -655,22 +655,22 @@
         <v>15</v>
       </c>
       <c r="B10">
-        <v>1543</v>
+        <v>1619</v>
       </c>
       <c r="C10">
-        <v>1486</v>
+        <v>1500</v>
       </c>
       <c r="D10">
-        <v>9700</v>
+        <v>10845</v>
       </c>
       <c r="E10">
-        <v>1272</v>
+        <v>1283</v>
       </c>
       <c r="F10">
-        <v>85.59999999999999</v>
+        <v>85.5</v>
       </c>
       <c r="G10">
-        <v>217154</v>
+        <v>211863</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -678,22 +678,22 @@
         <v>16</v>
       </c>
       <c r="B11">
-        <v>991</v>
+        <v>997</v>
       </c>
       <c r="C11">
-        <v>876</v>
+        <v>840</v>
       </c>
       <c r="D11">
-        <v>5715</v>
+        <v>5831</v>
       </c>
       <c r="E11">
-        <v>777</v>
+        <v>743</v>
       </c>
       <c r="F11">
-        <v>88.7</v>
+        <v>88.5</v>
       </c>
       <c r="G11">
-        <v>138970</v>
+        <v>135987</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -701,22 +701,22 @@
         <v>17</v>
       </c>
       <c r="B12">
-        <v>1122</v>
+        <v>1127</v>
       </c>
       <c r="C12">
-        <v>571</v>
+        <v>560</v>
       </c>
       <c r="D12">
-        <v>6524</v>
+        <v>6604</v>
       </c>
       <c r="E12">
-        <v>517</v>
+        <v>506</v>
       </c>
       <c r="F12">
-        <v>90.5</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="G12">
-        <v>71155</v>
+        <v>69866</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -727,19 +727,19 @@
         <v>3753</v>
       </c>
       <c r="C13">
-        <v>2975</v>
+        <v>2937</v>
       </c>
       <c r="D13">
         <v>21939</v>
       </c>
       <c r="E13">
-        <v>2149</v>
+        <v>2115</v>
       </c>
       <c r="F13">
-        <v>72.2</v>
+        <v>72</v>
       </c>
       <c r="G13">
-        <v>51505</v>
+        <v>49603</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -750,19 +750,19 @@
         <v>2402</v>
       </c>
       <c r="C14">
-        <v>1760</v>
+        <v>1739</v>
       </c>
       <c r="D14">
         <v>14293</v>
       </c>
       <c r="E14">
-        <v>1235</v>
+        <v>1219</v>
       </c>
       <c r="F14">
-        <v>70.2</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="G14">
-        <v>37127</v>
+        <v>36920</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -773,19 +773,19 @@
         <v>2077</v>
       </c>
       <c r="C15">
-        <v>519</v>
+        <v>507</v>
       </c>
       <c r="D15">
         <v>17453</v>
       </c>
       <c r="E15">
-        <v>447</v>
+        <v>435</v>
       </c>
       <c r="F15">
-        <v>86.09999999999999</v>
+        <v>85.8</v>
       </c>
       <c r="G15">
-        <v>23899</v>
+        <v>23697</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -793,22 +793,22 @@
         <v>21</v>
       </c>
       <c r="B16">
-        <v>1039</v>
+        <v>1045</v>
       </c>
       <c r="C16">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="D16">
-        <v>6274</v>
+        <v>6328</v>
       </c>
       <c r="E16">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="F16">
-        <v>87.3</v>
+        <v>87.2</v>
       </c>
       <c r="G16">
-        <v>13188</v>
+        <v>13130</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -816,19 +816,19 @@
         <v>22</v>
       </c>
       <c r="B17">
-        <v>2549</v>
+        <v>2552</v>
       </c>
       <c r="C17">
-        <v>871</v>
+        <v>854</v>
       </c>
       <c r="D17">
-        <v>18216</v>
+        <v>18243</v>
       </c>
       <c r="E17">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="F17">
-        <v>23.3</v>
+        <v>23.2</v>
       </c>
       <c r="G17">
         <v>639</v>

</xml_diff>

<commit_message>
daily auto-refresh 2026-10-23 11:02
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,120 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>sample_orders</t>
-  </si>
-  <si>
-    <t>new_creators</t>
-  </si>
-  <si>
-    <t>cogs</t>
-  </si>
-  <si>
-    <t>posted</t>
-  </si>
-  <si>
-    <t>post_rate</t>
-  </si>
-  <si>
-    <t>video_gmv</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
-  </si>
-  <si>
-    <t>2026-01</t>
-  </si>
-  <si>
-    <t>2026-02</t>
-  </si>
-  <si>
-    <t>2026-03</t>
-  </si>
-  <si>
-    <t>2026-04</t>
-  </si>
-  <si>
-    <t>2026-05</t>
-  </si>
-  <si>
-    <t>2026-06</t>
-  </si>
-  <si>
-    <t>2026-07</t>
-  </si>
-  <si>
-    <t>2026-08</t>
-  </si>
-  <si>
-    <t>2026-09</t>
-  </si>
-  <si>
-    <t>2026-10</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -122,36 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -439,402 +408,452 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sample_orders</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>new_creators</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cogs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>posted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>post_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>video_gmv</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>73</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>70</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>415</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>59</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>84.3</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>17413</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>42</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>41</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>243</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>33</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>80.5</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>18234</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>442</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>433</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>2539</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>298</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>68.8</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>214755</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>662</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>605</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>3865</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>386</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>63.8</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>46738</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>765</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>715</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>4498</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>421</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>58.9</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>85640</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>531</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>491</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>3138</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>313</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>63.7</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>27811</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>979</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>924</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>6589</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>546</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>59.1</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>62714</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1113</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>997</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>9651</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>788</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>79</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>67643</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>1619</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>1500</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>10845</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>1283</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>85.5</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>211865</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>997</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>840</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>5831</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>743</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>88.5</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>135988</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1127</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="n">
         <v>560</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>6604</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>506</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="n">
         <v>69868</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>3753</v>
       </c>
-      <c r="C13">
+      <c r="C13" t="n">
         <v>2937</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>21939</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>2115</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>72</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>49604</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>2402</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="n">
         <v>1739</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>14293</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>1219</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>70.09999999999999</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>36921</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>2077</v>
       </c>
-      <c r="C15">
+      <c r="C15" t="n">
         <v>507</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>17453</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>435</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>85.8</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>23699</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>1045</v>
       </c>
-      <c r="C16">
+      <c r="C16" t="n">
         <v>329</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>6328</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>287</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="n">
         <v>87.2</v>
       </c>
-      <c r="G16">
+      <c r="G16" t="n">
         <v>13130</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17">
-        <v>2552</v>
-      </c>
-      <c r="C17">
-        <v>854</v>
-      </c>
-      <c r="D17">
-        <v>18243</v>
-      </c>
-      <c r="E17">
-        <v>201</v>
-      </c>
-      <c r="F17">
-        <v>23.5</v>
-      </c>
-      <c r="G17">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>2767</v>
+      </c>
+      <c r="C17" t="n">
+        <v>935</v>
+      </c>
+      <c r="D17" t="n">
+        <v>19660</v>
+      </c>
+      <c r="E17" t="n">
+        <v>200</v>
+      </c>
+      <c r="F17" t="n">
+        <v>21.4</v>
+      </c>
+      <c r="G17" t="n">
         <v>639</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-23 06:17
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,452 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>415</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>59</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>84.3</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17413</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>243</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18234</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>442</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>433</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2539</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>298</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>214755</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>662</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>605</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3865</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>386</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>63.8</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>46738</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>765</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>715</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>4498</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>421</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>58.9</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>85640</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>531</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>491</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>3138</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>313</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>63.7</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>27811</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>979</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>924</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>6589</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>546</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>59.1</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>62714</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>1113</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>997</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>9651</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>788</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>79</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>67643</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1619</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1500</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>10845</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1283</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>85.5</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>211865</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>997</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>840</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>5831</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>743</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>88.5</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>135988</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1127</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>560</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6604</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>506</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>69868</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3753</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>2937</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>21939</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2115</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>72</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>49604</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>2402</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>1739</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>14293</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1219</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>70.09999999999999</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>36921</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2077</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>507</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>17453</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>435</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>85.8</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>23699</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1045</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>329</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>6328</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>287</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>87.2</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>13130</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
         <v>2767</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>935</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17">
         <v>19660</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>200</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17">
         <v>21.4</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17">
         <v>639</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-26 07:22
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,452 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>415</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>59</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>84.3</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17476</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>243</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18208</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>442</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>433</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2539</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>298</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>214943</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>662</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>605</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3865</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>386</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>63.8</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>46824</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>765</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>715</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>4498</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>421</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>58.9</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>85938</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>531</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>491</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>3138</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>313</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>63.7</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>28000</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>979</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>924</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>6589</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>546</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>59.1</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>62479</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>1113</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>997</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>9651</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>788</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>79</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>67699</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1619</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1500</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>10845</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1283</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>85.5</v>
       </c>
-      <c r="G10" t="n">
-        <v>213071</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+      <c r="G10">
+        <v>213068</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>997</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>840</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>5831</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>743</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>88.5</v>
       </c>
-      <c r="G11" t="n">
-        <v>136030</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+      <c r="G11">
+        <v>136032</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1127</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>560</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6604</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>506</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12" t="n">
-        <v>69916</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+      <c r="G12">
+        <v>69915</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3753</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>2937</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>21939</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2115</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>72</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>49530</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>2402</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>1739</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>14293</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1219</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>70.09999999999999</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>37667</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2077</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>507</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>17453</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>435</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>85.8</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>23718</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1045</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>329</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>6328</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>287</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>87.2</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>13545</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>2766</v>
-      </c>
-      <c r="C17" t="n">
-        <v>934</v>
-      </c>
-      <c r="D17" t="n">
-        <v>19655</v>
-      </c>
-      <c r="E17" t="n">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>3165</v>
+      </c>
+      <c r="C17">
+        <v>1112</v>
+      </c>
+      <c r="D17">
+        <v>22093</v>
+      </c>
+      <c r="E17">
         <v>256</v>
       </c>
-      <c r="F17" t="n">
-        <v>27.4</v>
-      </c>
-      <c r="G17" t="n">
+      <c r="F17">
+        <v>23</v>
+      </c>
+      <c r="G17">
         <v>920</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-26 13:04
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,120 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>sample_orders</t>
-  </si>
-  <si>
-    <t>new_creators</t>
-  </si>
-  <si>
-    <t>cogs</t>
-  </si>
-  <si>
-    <t>posted</t>
-  </si>
-  <si>
-    <t>post_rate</t>
-  </si>
-  <si>
-    <t>video_gmv</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
-  </si>
-  <si>
-    <t>2026-01</t>
-  </si>
-  <si>
-    <t>2026-02</t>
-  </si>
-  <si>
-    <t>2026-03</t>
-  </si>
-  <si>
-    <t>2026-04</t>
-  </si>
-  <si>
-    <t>2026-05</t>
-  </si>
-  <si>
-    <t>2026-06</t>
-  </si>
-  <si>
-    <t>2026-07</t>
-  </si>
-  <si>
-    <t>2026-08</t>
-  </si>
-  <si>
-    <t>2026-09</t>
-  </si>
-  <si>
-    <t>2026-10</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -122,36 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -439,402 +408,452 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sample_orders</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>new_creators</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cogs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>posted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>post_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>video_gmv</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>73</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>70</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>415</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>59</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>84.3</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>17476</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>42</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>41</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>243</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>33</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>80.5</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>18208</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>442</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>433</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>2539</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>298</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>68.8</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>214943</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>662</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>605</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>3865</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>386</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>63.8</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>46824</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>765</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>715</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>4498</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>421</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>58.9</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>85938</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>531</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>491</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>3138</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>313</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>63.7</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>28000</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>979</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>924</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>6589</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>546</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>59.1</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>62479</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1113</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>997</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>9651</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>788</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>79</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>67699</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>1619</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>1500</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>10845</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>1283</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>85.5</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>213068</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>997</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>840</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>5831</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>743</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>88.5</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>136032</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1127</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="n">
         <v>560</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>6604</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>506</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="n">
         <v>69915</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>3753</v>
       </c>
-      <c r="C13">
+      <c r="C13" t="n">
         <v>2937</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>21939</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>2115</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>72</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>49530</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>2402</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="n">
         <v>1739</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>14293</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>1219</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>70.09999999999999</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>37667</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>2077</v>
       </c>
-      <c r="C15">
+      <c r="C15" t="n">
         <v>507</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>17453</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>435</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>85.8</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>23718</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>1045</v>
       </c>
-      <c r="C16">
+      <c r="C16" t="n">
         <v>329</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>6328</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>287</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="n">
         <v>87.2</v>
       </c>
-      <c r="G16">
+      <c r="G16" t="n">
         <v>13545</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>3165</v>
       </c>
-      <c r="C17">
+      <c r="C17" t="n">
         <v>1112</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="n">
         <v>22093</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="n">
         <v>256</v>
       </c>
-      <c r="F17">
+      <c r="F17" t="n">
         <v>23</v>
       </c>
-      <c r="G17">
+      <c r="G17" t="n">
         <v>920</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-26 07:47
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,452 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>415</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>59</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>84.3</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17476</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>243</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18208</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>442</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>433</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2539</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>298</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>214943</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>662</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>605</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3865</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>386</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>63.8</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>46824</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>765</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>715</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>4498</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>421</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>58.9</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>85938</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>531</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>491</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>3138</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>313</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>63.7</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>28000</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>979</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>924</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>6589</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>546</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>59.1</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>62479</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>1113</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>997</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>9651</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>788</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>79</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>67699</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1619</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1500</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>10845</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1283</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>85.5</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>213068</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>997</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>840</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>5831</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>743</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>88.5</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>136032</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1127</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>560</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6604</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>506</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>69915</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3753</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>2937</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>21939</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2115</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>72</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>49530</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>2402</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>1739</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>14293</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1219</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>70.09999999999999</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>37667</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2077</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>507</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>17453</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>435</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>85.8</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>23718</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1045</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>329</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>6328</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>287</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>87.2</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>13545</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
         <v>3165</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>1112</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17">
         <v>22093</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>256</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17">
         <v>23</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17">
         <v>920</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-26 15:04
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,120 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>sample_orders</t>
-  </si>
-  <si>
-    <t>new_creators</t>
-  </si>
-  <si>
-    <t>cogs</t>
-  </si>
-  <si>
-    <t>posted</t>
-  </si>
-  <si>
-    <t>post_rate</t>
-  </si>
-  <si>
-    <t>video_gmv</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
-  </si>
-  <si>
-    <t>2026-01</t>
-  </si>
-  <si>
-    <t>2026-02</t>
-  </si>
-  <si>
-    <t>2026-03</t>
-  </si>
-  <si>
-    <t>2026-04</t>
-  </si>
-  <si>
-    <t>2026-05</t>
-  </si>
-  <si>
-    <t>2026-06</t>
-  </si>
-  <si>
-    <t>2026-07</t>
-  </si>
-  <si>
-    <t>2026-08</t>
-  </si>
-  <si>
-    <t>2026-09</t>
-  </si>
-  <si>
-    <t>2026-10</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -122,36 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -439,402 +408,452 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sample_orders</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>new_creators</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cogs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>posted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>post_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>video_gmv</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>73</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>70</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>415</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>59</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>84.3</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>17491</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>42</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>41</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>243</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>33</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>80.5</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>18208</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>442</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>433</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>2539</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>298</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>68.8</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>214705</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>662</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>605</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>3865</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>386</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>63.8</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>46996</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>765</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>715</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>4498</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>421</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>58.9</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>85853</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>531</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>491</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>3138</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>313</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>63.7</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>28426</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>979</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>924</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>6589</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>547</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>59.2</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>61743</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1113</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>997</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>9651</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>788</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>79</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>67740</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>1619</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>1500</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>10845</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>1284</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>85.59999999999999</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>214891</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>997</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>840</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>5831</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>744</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>88.59999999999999</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>136288</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1127</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="n">
         <v>560</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>6604</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>506</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="n">
         <v>69522</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>3753</v>
       </c>
-      <c r="C13">
+      <c r="C13" t="n">
         <v>2937</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>21939</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>2115</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>72</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>49261</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>2402</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="n">
         <v>1739</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>14293</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>1218</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>70</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>38890</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>2077</v>
       </c>
-      <c r="C15">
+      <c r="C15" t="n">
         <v>507</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>17453</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>436</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>86</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>23451</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>1045</v>
       </c>
-      <c r="C16">
+      <c r="C16" t="n">
         <v>329</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>6328</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>288</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="n">
         <v>87.5</v>
       </c>
-      <c r="G16">
+      <c r="G16" t="n">
         <v>14013</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
         <v>3165</v>
       </c>
-      <c r="C17">
+      <c r="C17" t="n">
         <v>1112</v>
       </c>
-      <c r="D17">
+      <c r="D17" t="n">
         <v>22093</v>
       </c>
-      <c r="E17">
+      <c r="E17" t="n">
         <v>384</v>
       </c>
-      <c r="F17">
+      <c r="F17" t="n">
         <v>34.5</v>
       </c>
-      <c r="G17">
+      <c r="G17" t="n">
         <v>1471</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-26 09:52
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,452 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>415</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>59</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>84.3</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17491</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>243</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18208</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>442</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>433</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2539</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>298</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>214705</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>662</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>605</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3865</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>386</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>63.8</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>46996</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>765</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>715</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>4498</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>421</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>58.9</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>85853</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>531</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>491</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>3138</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>313</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>63.7</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>28426</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>979</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>924</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>6589</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>547</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>59.2</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>61743</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>1113</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>997</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>9651</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>788</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>79</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>67740</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1619</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1500</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>10845</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1284</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>85.59999999999999</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>214891</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>997</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>840</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>5831</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>744</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>88.59999999999999</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>136288</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1127</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>560</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6604</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>506</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>69522</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3753</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>2937</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>21939</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2115</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>72</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>49261</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>2402</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>1739</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>14293</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1218</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>70</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>38890</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2077</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>507</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>17453</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>436</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>86</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>23451</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1045</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>329</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>6328</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>288</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>87.5</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>14013</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
         <v>3165</v>
       </c>
-      <c r="C17" t="n">
+      <c r="C17">
         <v>1112</v>
       </c>
-      <c r="D17" t="n">
+      <c r="D17">
         <v>22093</v>
       </c>
-      <c r="E17" t="n">
+      <c r="E17">
         <v>384</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17">
         <v>34.5</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17">
         <v>1471</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-27 11:46
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,120 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
-  <workbookPr defaultThemeVersion="124226"/>
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
-  <si>
-    <t>month</t>
-  </si>
-  <si>
-    <t>sample_orders</t>
-  </si>
-  <si>
-    <t>new_creators</t>
-  </si>
-  <si>
-    <t>cogs</t>
-  </si>
-  <si>
-    <t>posted</t>
-  </si>
-  <si>
-    <t>post_rate</t>
-  </si>
-  <si>
-    <t>video_gmv</t>
-  </si>
-  <si>
-    <t>2025-07</t>
-  </si>
-  <si>
-    <t>2025-08</t>
-  </si>
-  <si>
-    <t>2025-09</t>
-  </si>
-  <si>
-    <t>2025-10</t>
-  </si>
-  <si>
-    <t>2025-11</t>
-  </si>
-  <si>
-    <t>2025-12</t>
-  </si>
-  <si>
-    <t>2026-01</t>
-  </si>
-  <si>
-    <t>2026-02</t>
-  </si>
-  <si>
-    <t>2026-03</t>
-  </si>
-  <si>
-    <t>2026-04</t>
-  </si>
-  <si>
-    <t>2026-05</t>
-  </si>
-  <si>
-    <t>2026-06</t>
-  </si>
-  <si>
-    <t>2026-07</t>
-  </si>
-  <si>
-    <t>2026-08</t>
-  </si>
-  <si>
-    <t>2026-09</t>
-  </si>
-  <si>
-    <t>2026-10</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <numFmts count="0"/>
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <color theme="1"/>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -122,36 +42,85 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+  <cellXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -439,402 +408,452 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G17"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:7">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>month</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sample_orders</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>new_creators</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>cogs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>posted</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>post_rate</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>video_gmv</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
         <v>73</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="n">
         <v>70</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="n">
         <v>415</v>
       </c>
-      <c r="E2">
+      <c r="E2" t="n">
         <v>59</v>
       </c>
-      <c r="F2">
+      <c r="F2" t="n">
         <v>84.3</v>
       </c>
-      <c r="G2">
+      <c r="G2" t="n">
         <v>17491</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3">
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>42</v>
       </c>
-      <c r="C3">
+      <c r="C3" t="n">
         <v>41</v>
       </c>
-      <c r="D3">
+      <c r="D3" t="n">
         <v>243</v>
       </c>
-      <c r="E3">
+      <c r="E3" t="n">
         <v>33</v>
       </c>
-      <c r="F3">
+      <c r="F3" t="n">
         <v>80.5</v>
       </c>
-      <c r="G3">
+      <c r="G3" t="n">
         <v>18208</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4">
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
         <v>442</v>
       </c>
-      <c r="C4">
+      <c r="C4" t="n">
         <v>433</v>
       </c>
-      <c r="D4">
+      <c r="D4" t="n">
         <v>2539</v>
       </c>
-      <c r="E4">
+      <c r="E4" t="n">
         <v>298</v>
       </c>
-      <c r="F4">
+      <c r="F4" t="n">
         <v>68.8</v>
       </c>
-      <c r="G4">
+      <c r="G4" t="n">
         <v>214705</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
-      <c r="A5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5">
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
         <v>662</v>
       </c>
-      <c r="C5">
+      <c r="C5" t="n">
         <v>605</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="n">
         <v>3865</v>
       </c>
-      <c r="E5">
+      <c r="E5" t="n">
         <v>386</v>
       </c>
-      <c r="F5">
+      <c r="F5" t="n">
         <v>63.8</v>
       </c>
-      <c r="G5">
+      <c r="G5" t="n">
         <v>46996</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
-      <c r="A6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6">
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>765</v>
       </c>
-      <c r="C6">
+      <c r="C6" t="n">
         <v>715</v>
       </c>
-      <c r="D6">
+      <c r="D6" t="n">
         <v>4498</v>
       </c>
-      <c r="E6">
+      <c r="E6" t="n">
         <v>421</v>
       </c>
-      <c r="F6">
+      <c r="F6" t="n">
         <v>58.9</v>
       </c>
-      <c r="G6">
+      <c r="G6" t="n">
         <v>85853</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7">
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
         <v>531</v>
       </c>
-      <c r="C7">
+      <c r="C7" t="n">
         <v>491</v>
       </c>
-      <c r="D7">
+      <c r="D7" t="n">
         <v>3138</v>
       </c>
-      <c r="E7">
+      <c r="E7" t="n">
         <v>313</v>
       </c>
-      <c r="F7">
+      <c r="F7" t="n">
         <v>63.7</v>
       </c>
-      <c r="G7">
+      <c r="G7" t="n">
         <v>28426</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8">
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
         <v>979</v>
       </c>
-      <c r="C8">
+      <c r="C8" t="n">
         <v>924</v>
       </c>
-      <c r="D8">
+      <c r="D8" t="n">
         <v>6589</v>
       </c>
-      <c r="E8">
+      <c r="E8" t="n">
         <v>547</v>
       </c>
-      <c r="F8">
+      <c r="F8" t="n">
         <v>59.2</v>
       </c>
-      <c r="G8">
+      <c r="G8" t="n">
         <v>61743</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
         <v>1113</v>
       </c>
-      <c r="C9">
+      <c r="C9" t="n">
         <v>997</v>
       </c>
-      <c r="D9">
+      <c r="D9" t="n">
         <v>9651</v>
       </c>
-      <c r="E9">
+      <c r="E9" t="n">
         <v>788</v>
       </c>
-      <c r="F9">
+      <c r="F9" t="n">
         <v>79</v>
       </c>
-      <c r="G9">
+      <c r="G9" t="n">
         <v>67740</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10">
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
         <v>1619</v>
       </c>
-      <c r="C10">
+      <c r="C10" t="n">
         <v>1500</v>
       </c>
-      <c r="D10">
+      <c r="D10" t="n">
         <v>10845</v>
       </c>
-      <c r="E10">
+      <c r="E10" t="n">
         <v>1284</v>
       </c>
-      <c r="F10">
+      <c r="F10" t="n">
         <v>85.59999999999999</v>
       </c>
-      <c r="G10">
+      <c r="G10" t="n">
         <v>214891</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
-      <c r="A11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11">
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
         <v>997</v>
       </c>
-      <c r="C11">
+      <c r="C11" t="n">
         <v>840</v>
       </c>
-      <c r="D11">
+      <c r="D11" t="n">
         <v>5831</v>
       </c>
-      <c r="E11">
+      <c r="E11" t="n">
         <v>744</v>
       </c>
-      <c r="F11">
+      <c r="F11" t="n">
         <v>88.59999999999999</v>
       </c>
-      <c r="G11">
+      <c r="G11" t="n">
         <v>136288</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
-      <c r="A12" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12">
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
         <v>1127</v>
       </c>
-      <c r="C12">
+      <c r="C12" t="n">
         <v>560</v>
       </c>
-      <c r="D12">
+      <c r="D12" t="n">
         <v>6604</v>
       </c>
-      <c r="E12">
+      <c r="E12" t="n">
         <v>506</v>
       </c>
-      <c r="F12">
+      <c r="F12" t="n">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12">
+      <c r="G12" t="n">
         <v>69522</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
-      <c r="A13" t="s">
-        <v>18</v>
-      </c>
-      <c r="B13">
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
         <v>3753</v>
       </c>
-      <c r="C13">
+      <c r="C13" t="n">
         <v>2937</v>
       </c>
-      <c r="D13">
+      <c r="D13" t="n">
         <v>21939</v>
       </c>
-      <c r="E13">
+      <c r="E13" t="n">
         <v>2115</v>
       </c>
-      <c r="F13">
+      <c r="F13" t="n">
         <v>72</v>
       </c>
-      <c r="G13">
+      <c r="G13" t="n">
         <v>49261</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
-      <c r="A14" t="s">
-        <v>19</v>
-      </c>
-      <c r="B14">
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
         <v>2402</v>
       </c>
-      <c r="C14">
+      <c r="C14" t="n">
         <v>1739</v>
       </c>
-      <c r="D14">
+      <c r="D14" t="n">
         <v>14293</v>
       </c>
-      <c r="E14">
+      <c r="E14" t="n">
         <v>1218</v>
       </c>
-      <c r="F14">
+      <c r="F14" t="n">
         <v>70</v>
       </c>
-      <c r="G14">
+      <c r="G14" t="n">
         <v>38890</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
-      <c r="A15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B15">
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>2077</v>
       </c>
-      <c r="C15">
+      <c r="C15" t="n">
         <v>507</v>
       </c>
-      <c r="D15">
+      <c r="D15" t="n">
         <v>17453</v>
       </c>
-      <c r="E15">
+      <c r="E15" t="n">
         <v>436</v>
       </c>
-      <c r="F15">
+      <c r="F15" t="n">
         <v>86</v>
       </c>
-      <c r="G15">
+      <c r="G15" t="n">
         <v>23451</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
-      <c r="A16" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16">
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
         <v>1045</v>
       </c>
-      <c r="C16">
+      <c r="C16" t="n">
         <v>329</v>
       </c>
-      <c r="D16">
+      <c r="D16" t="n">
         <v>6328</v>
       </c>
-      <c r="E16">
+      <c r="E16" t="n">
         <v>288</v>
       </c>
-      <c r="F16">
+      <c r="F16" t="n">
         <v>87.5</v>
       </c>
-      <c r="G16">
+      <c r="G16" t="n">
         <v>14013</v>
       </c>
     </row>
-    <row r="17" spans="1:7">
-      <c r="A17" t="s">
-        <v>22</v>
-      </c>
-      <c r="B17">
-        <v>3165</v>
-      </c>
-      <c r="C17">
-        <v>1112</v>
-      </c>
-      <c r="D17">
-        <v>22093</v>
-      </c>
-      <c r="E17">
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3303</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1164</v>
+      </c>
+      <c r="D17" t="n">
+        <v>23028</v>
+      </c>
+      <c r="E17" t="n">
         <v>384</v>
       </c>
-      <c r="F17">
-        <v>34.5</v>
-      </c>
-      <c r="G17">
+      <c r="F17" t="n">
+        <v>33</v>
+      </c>
+      <c r="G17" t="n">
         <v>1471</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-27 06:44
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,452 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>415</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>59</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>84.3</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17491</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>243</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18208</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>442</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>433</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2539</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>298</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>214705</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>662</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>605</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3865</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>386</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>63.8</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>46996</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>765</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>715</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>4498</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>421</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>58.9</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>85853</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>531</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>491</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>3138</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>313</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>63.7</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>28426</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>979</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>924</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>6589</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>547</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>59.2</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>61743</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>1113</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>997</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>9651</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>788</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>79</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>67740</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1619</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1500</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>10845</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1284</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>85.59999999999999</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>214891</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>997</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>840</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>5831</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>744</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>88.59999999999999</v>
       </c>
-      <c r="G11" t="n">
+      <c r="G11">
         <v>136288</v>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1127</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>560</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6604</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>506</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>69522</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3753</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>2937</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>21939</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2115</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>72</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>49261</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>2402</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>1739</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>14293</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1218</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>70</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>38890</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2077</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>507</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>17453</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>436</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>86</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>23451</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1045</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>329</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>6328</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>288</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>87.5</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>14013</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>3303</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1164</v>
-      </c>
-      <c r="D17" t="n">
-        <v>23028</v>
-      </c>
-      <c r="E17" t="n">
-        <v>384</v>
-      </c>
-      <c r="F17" t="n">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>3300</v>
+      </c>
+      <c r="C17">
+        <v>1162</v>
+      </c>
+      <c r="D17">
+        <v>23010</v>
+      </c>
+      <c r="E17">
+        <v>383</v>
+      </c>
+      <c r="F17">
         <v>33</v>
       </c>
-      <c r="G17" t="n">
+      <c r="G17">
         <v>1471</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
daily auto-refresh 2026-10-28 06:43
</commit_message>
<xml_diff>
--- a/monthly_sample_report.xlsx
+++ b/monthly_sample_report.xlsx
@@ -1,40 +1,120 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <workbookPr/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+  <si>
+    <t>month</t>
+  </si>
+  <si>
+    <t>sample_orders</t>
+  </si>
+  <si>
+    <t>new_creators</t>
+  </si>
+  <si>
+    <t>cogs</t>
+  </si>
+  <si>
+    <t>posted</t>
+  </si>
+  <si>
+    <t>post_rate</t>
+  </si>
+  <si>
+    <t>video_gmv</t>
+  </si>
+  <si>
+    <t>2025-07</t>
+  </si>
+  <si>
+    <t>2025-08</t>
+  </si>
+  <si>
+    <t>2025-09</t>
+  </si>
+  <si>
+    <t>2025-10</t>
+  </si>
+  <si>
+    <t>2025-11</t>
+  </si>
+  <si>
+    <t>2025-12</t>
+  </si>
+  <si>
+    <t>2026-01</t>
+  </si>
+  <si>
+    <t>2026-02</t>
+  </si>
+  <si>
+    <t>2026-03</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2026-05</t>
+  </si>
+  <si>
+    <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
+  </si>
+  <si>
+    <t>2026-08</t>
+  </si>
+  <si>
+    <t>2026-09</t>
+  </si>
+  <si>
+    <t>2026-10</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,85 +122,36 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -408,452 +439,402 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>month</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>sample_orders</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>new_creators</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>cogs</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>posted</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>post_rate</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>video_gmv</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>2025-07</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+    <row r="1" spans="1:7">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
         <v>73</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C2">
         <v>70</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D2">
         <v>415</v>
       </c>
-      <c r="E2" t="n">
+      <c r="E2">
         <v>59</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2">
         <v>84.3</v>
       </c>
-      <c r="G2" t="n">
+      <c r="G2">
         <v>17501</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>2025-08</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
         <v>42</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3">
         <v>41</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3">
         <v>243</v>
       </c>
-      <c r="E3" t="n">
+      <c r="E3">
         <v>33</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3">
         <v>80.5</v>
       </c>
-      <c r="G3" t="n">
+      <c r="G3">
         <v>18208</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>2025-09</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
         <v>442</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4">
         <v>433</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4">
         <v>2539</v>
       </c>
-      <c r="E4" t="n">
+      <c r="E4">
         <v>298</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4">
         <v>68.8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="G4">
         <v>214686</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>2025-10</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
         <v>662</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5">
         <v>605</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5">
         <v>3865</v>
       </c>
-      <c r="E5" t="n">
+      <c r="E5">
         <v>386</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5">
         <v>63.8</v>
       </c>
-      <c r="G5" t="n">
+      <c r="G5">
         <v>47030</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2025-11</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
         <v>765</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6">
         <v>715</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6">
         <v>4498</v>
       </c>
-      <c r="E6" t="n">
+      <c r="E6">
         <v>421</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6">
         <v>58.9</v>
       </c>
-      <c r="G6" t="n">
+      <c r="G6">
         <v>85847</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>2025-12</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
         <v>531</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7">
         <v>491</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7">
         <v>3138</v>
       </c>
-      <c r="E7" t="n">
+      <c r="E7">
         <v>313</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7">
         <v>63.7</v>
       </c>
-      <c r="G7" t="n">
+      <c r="G7">
         <v>28573</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>2026-01</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
         <v>979</v>
       </c>
-      <c r="C8" t="n">
+      <c r="C8">
         <v>924</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8">
         <v>6589</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E8">
         <v>547</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8">
         <v>59.2</v>
       </c>
-      <c r="G8" t="n">
+      <c r="G8">
         <v>61565</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2026-02</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
         <v>1113</v>
       </c>
-      <c r="C9" t="n">
+      <c r="C9">
         <v>997</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9">
         <v>9651</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E9">
         <v>788</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9">
         <v>79</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G9">
         <v>67808</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-03</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
         <v>1619</v>
       </c>
-      <c r="C10" t="n">
+      <c r="C10">
         <v>1500</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10">
         <v>10845</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E10">
         <v>1284</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10">
         <v>85.59999999999999</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G10">
         <v>215047</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-04</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
         <v>997</v>
       </c>
-      <c r="C11" t="n">
+      <c r="C11">
         <v>840</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11">
         <v>5831</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E11">
         <v>744</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11">
         <v>88.59999999999999</v>
       </c>
-      <c r="G11" t="n">
-        <v>136319</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-05</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
+      <c r="G11">
+        <v>136317</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12">
         <v>1127</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C12">
         <v>560</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12">
         <v>6604</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E12">
         <v>506</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12">
         <v>90.40000000000001</v>
       </c>
-      <c r="G12" t="n">
+      <c r="G12">
         <v>69635</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-06</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13">
         <v>3753</v>
       </c>
-      <c r="C13" t="n">
+      <c r="C13">
         <v>2937</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13">
         <v>21939</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E13">
         <v>2115</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13">
         <v>72</v>
       </c>
-      <c r="G13" t="n">
+      <c r="G13">
         <v>49044</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14">
         <v>2402</v>
       </c>
-      <c r="C14" t="n">
+      <c r="C14">
         <v>1739</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14">
         <v>14293</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E14">
         <v>1218</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14">
         <v>70</v>
       </c>
-      <c r="G14" t="n">
+      <c r="G14">
         <v>39293</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15">
         <v>2077</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C15">
         <v>507</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15">
         <v>17453</v>
       </c>
-      <c r="E15" t="n">
+      <c r="E15">
         <v>437</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15">
         <v>86.2</v>
       </c>
-      <c r="G15" t="n">
+      <c r="G15">
         <v>23145</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
+        <v>21</v>
+      </c>
+      <c r="B16">
         <v>1045</v>
       </c>
-      <c r="C16" t="n">
+      <c r="C16">
         <v>329</v>
       </c>
-      <c r="D16" t="n">
+      <c r="D16">
         <v>6328</v>
       </c>
-      <c r="E16" t="n">
+      <c r="E16">
         <v>288</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16">
         <v>87.5</v>
       </c>
-      <c r="G16" t="n">
+      <c r="G16">
         <v>14362</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-10</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>3300</v>
-      </c>
-      <c r="C17" t="n">
-        <v>1162</v>
-      </c>
-      <c r="D17" t="n">
-        <v>23010</v>
-      </c>
-      <c r="E17" t="n">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17">
+        <v>3394</v>
+      </c>
+      <c r="C17">
+        <v>1198</v>
+      </c>
+      <c r="D17">
+        <v>23731</v>
+      </c>
+      <c r="E17">
         <v>412</v>
       </c>
-      <c r="F17" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="G17" t="n">
+      <c r="F17">
+        <v>34.4</v>
+      </c>
+      <c r="G17">
         <v>1931</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>